<commit_message>
Small edits to template functions.
</commit_message>
<xml_diff>
--- a/dev/test_small_new.xlsx
+++ b/dev/test_small_new.xlsx
@@ -26,12 +26,11 @@
   <si>
     <t xml:space="preserve">Welcome to the NCAI Data Entry Template. Complete the sheets with your own data as follows:
  Habitat extent: area of each habitat (e.g. in hectares) each year.
- Provision Per Unit: score, typically out of 5, representing the expemplary per unit provision of ecosystem services per unit of area. If scoring out of a different number, specify the divisor in get_ncai(). 
- Importance: define relative importance of ecosystem service types, and the specific ecosystems within them.
+ Provision Per Unit: score, typically out of 5, representing the exemplary per unit provision of ecosystem services per unit of area.
+ Importance: define relative importance of ecosystem service types, and the specific services within them.
  Condition Indicator Scores: raw scores of each condition indicator in each year.
- Indicator Directory: salience (between 0 and 1) of condition indicators in representing likely flow of services in each ecosystem service type. 
- Individual condition indicator relevance shets: binary values denoting whether a condition indicator is relevant for each combination of habitat/ecosystem service (1 = relevant; 0 = not relevant). 
-</t>
+ Indicator Directory: salience (between 0 and 1) of condition indicators.
+ Individual condition indicator relevance sheets: binary values (1 = relevant; 0 = not relevant).</t>
   </si>
   <si>
     <t xml:space="preserve">Habitat extent in hectares</t>
@@ -61,7 +60,7 @@
     <t xml:space="preserve">3.5. Existence &amp; bequest</t>
   </si>
   <si>
-    <t xml:space="preserve">Step 1: ecosystem service type (SEEA) section. The most important service type is assigned a value of 20, and the other two are assigned a value (between 0 and 20) in terms of their relative importance.</t>
+    <t xml:space="preserve">Step 1: ecosystem service type (SEEA) section.</t>
   </si>
   <si>
     <t xml:space="preserve">Type</t>
@@ -76,7 +75,7 @@
     <t xml:space="preserve">CULTURAL</t>
   </si>
   <si>
-    <t xml:space="preserve">Step 2: PROVISIONING services. The most important is assigned a value of 20, and the others are assigned a value in terms of their relative importance.</t>
+    <t xml:space="preserve">Step 2: PROVISIONING services.</t>
   </si>
   <si>
     <t xml:space="preserve">Service</t>
@@ -85,7 +84,7 @@
     <t xml:space="preserve">Raw_Score</t>
   </si>
   <si>
-    <t xml:space="preserve">Step 2: CULTURAL services. The most important is assigned a value of 20, and the others are assigned a value in terms of their relative importance.</t>
+    <t xml:space="preserve">Step 2: CULTURAL services.</t>
   </si>
   <si>
     <t xml:space="preserve">Year</t>
@@ -100,7 +99,7 @@
     <t xml:space="preserve">Condition Indicator</t>
   </si>
   <si>
-    <t xml:space="preserve">Enter 1 or 0 in each cell of the matrix to denote whether this condition indicator is relevant in gauging flow.</t>
+    <t xml:space="preserve">Enter 1 or 0 in each cell.</t>
   </si>
 </sst>
 </file>
@@ -108,7 +107,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -139,20 +138,14 @@
       <b/>
     </font>
     <font>
-      <sz val="9"/>
-      <color rgb="FF000000"/>
+      <sz val="10"/>
+      <color rgb="FF0070C0"/>
       <name val="Calibri"/>
       <b/>
     </font>
     <font>
       <sz val="9"/>
-      <color rgb="FF0070C0"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF0070C0"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <b/>
     </font>
@@ -249,7 +242,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -258,16 +251,24 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment textRotation="90" horizontal="center" vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -276,38 +277,41 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment textRotation="90" horizontal="center" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment textRotation="90" horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2807,6 +2811,7 @@
       <c r="T100" s="1"/>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" sheet="1"/>
   <mergeCells count="1">
     <mergeCell ref="B4:J30"/>
   </mergeCells>
@@ -2830,25 +2835,25 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="8" t="n">
+      <c r="B1" t="n">
         <v>2020</v>
       </c>
-      <c r="C1" s="8" t="n">
+      <c r="C1" t="n">
         <v>2021</v>
       </c>
-      <c r="D1" s="8" t="n">
+      <c r="D1" t="n">
         <v>2022</v>
       </c>
-      <c r="E1" s="8" t="n">
+      <c r="E1" t="n">
         <v>2023</v>
       </c>
-      <c r="F1" s="8" t="n">
+      <c r="F1" t="n">
         <v>2024</v>
       </c>
-      <c r="G1" s="8" t="n">
+      <c r="G1" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -2945,6 +2950,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" sheet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
@@ -2962,7 +2968,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="180" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="8" t="s">
         <v>7</v>
       </c>
       <c r="B1" s="9" t="s">
@@ -3032,6 +3038,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" sheet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
@@ -3047,7 +3054,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="8" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3063,7 +3070,7 @@
       <c r="A3" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="17" t="n">
+      <c r="B3" s="15" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3071,12 +3078,12 @@
       <c r="A4" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="17" t="n">
+      <c r="B4" s="15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="8" t="s">
         <v>16</v>
       </c>
     </row>
@@ -3092,7 +3099,7 @@
       <c r="A10" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="17" t="n">
+      <c r="B10" s="15" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3100,12 +3107,12 @@
       <c r="A11" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="17" t="n">
+      <c r="B11" s="15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="8" t="s">
         <v>19</v>
       </c>
     </row>
@@ -3121,11 +3128,12 @@
       <c r="A16" t="s">
         <v>10</v>
       </c>
-      <c r="B16" s="17" t="n">
+      <c r="B16" s="15" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" sheet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
@@ -3142,83 +3150,84 @@
   </cols>
   <sheetData>
     <row r="1" ht="180" customHeight="1">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="16" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="21" t="n">
+      <c r="A2" s="19" t="n">
         <v>2020</v>
       </c>
-      <c r="B2" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" s="20" t="n">
+      <c r="B2" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" s="18" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="21" t="n">
+      <c r="A3" s="19" t="n">
         <v>2021</v>
       </c>
-      <c r="B3" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C3" s="20" t="n">
+      <c r="B3" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="18" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="21" t="n">
+      <c r="A4" s="19" t="n">
         <v>2022</v>
       </c>
-      <c r="B4" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" s="20" t="n">
+      <c r="B4" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="18" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="n">
+      <c r="A5" s="19" t="n">
         <v>2023</v>
       </c>
-      <c r="B5" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" s="20" t="n">
+      <c r="B5" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="18" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="21" t="n">
+      <c r="A6" s="19" t="n">
         <v>2024</v>
       </c>
-      <c r="B6" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" s="20" t="n">
+      <c r="B6" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="18" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="n">
+      <c r="A7" s="19" t="n">
         <v>2025</v>
       </c>
-      <c r="B7" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" s="20" t="n">
+      <c r="B7" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="18" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" sheet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
@@ -3233,39 +3242,40 @@
   </cols>
   <sheetData>
     <row r="1" ht="180" customHeight="1">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="16" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" s="19" t="n">
+      <c r="B2" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="C3" s="20" t="n">
+      <c r="B3" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="18" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" sheet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
@@ -3283,7 +3293,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="180" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="8" t="s">
         <v>24</v>
       </c>
       <c r="B1" s="9" t="s">
@@ -3353,6 +3363,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" sheet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
@@ -3370,7 +3381,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="180" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="8" t="s">
         <v>24</v>
       </c>
       <c r="B1" s="9" t="s">
@@ -3440,6 +3451,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" sheet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>

</xml_diff>